<commit_message>
docs: marketing collateral, corporate-pitch toolkit, sunscreen + shadow studies
Bundle of in-progress reference docs:

  - docs/community/SUNSCREEN_GUIDE.md — member-facing sunscreen
    recommendations for outdoor-pool sessions.
  - docs/strategy/SHADOW_STUDIES.md — coach-shadowing programme outline.
  - docs/marketing/COHORT_ENROLLMENT_OUTREACH_LIST.csv,
    docs/marketing/CONTENT_CREATOR_SCHEDULE.csv — operational lists for
    enrollment outreach and the content-creator rota.
  - docs/marketing/CORPORATE_WELLNESS.md — refreshed B2B wellness pitch.
  - docs/marketing/corporate_pitch/ — full corporate-pitch toolkit:
    cover-message templates, source markdown, generated PDF, and the
    build script (build_pitch_pdf.py) that produces the PDF from
    PITCH_SOURCE.md.
  - Minor revs to swimbuddz_content_calendar.xlsx,
    swimbuddz_content_templates.docx, swimbuddz_social_media_playbook.docx.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/marketing/swimbuddz_content_calendar.xlsx
+++ b/docs/marketing/swimbuddz_content_calendar.xlsx
@@ -1027,7 +1027,7 @@
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Create Business account @swimbuddz
-Bio: "Nigeria's first swimming community. Learn. Train. Belong. 🏊"
+Bio: "the global swimming community starting in Lagos. Learn. Train. Belong. 🏊"
 Profile photo: logo
 Set up Highlights (empty for now)</t>
         </is>
@@ -1035,7 +1035,7 @@
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Create Business account @swimbuddz
-Bio: "Nigeria's first swimming community 🏊 Watch adults learn to swim"
+Bio: "the global swimming community starting in Lagos 🏊 Watch adults learn to swim"
 Profile photo: same logo</t>
         </is>
       </c>
@@ -1115,7 +1115,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>30s: "Nigeria's first swimming community" montage of best pool footage</t>
+          <t>30s: "the global swimming community starting in Lagos" montage of best pool footage</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2597,7 +2597,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>#SwimBuddz #SwimBuddzNG</t>
+          <t>#SwimBuddz</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>#SwimSquad #SwimCommunity #LagosSwimmers #NigeriaSwims</t>
+          <t>#SwimSquad #SwimCommunity #NigeriaSwims</t>
         </is>
       </c>
     </row>

</xml_diff>